<commit_message>
Restructure priority_list with coverage matrix + dictionary updates
priority_list.txt: prepend 8 new top sections (Active Task Board,
Extractor Architecture, Variable Coverage Matrix, Per-Extractor
Gaps, Per-Extractor Unique Coverage, Dictionary Alignment, Naming
Inconsistencies, Pipeline Status) for project tracking. All
historical dated TODO blocks preserved verbatim below.

Coverage matrix verified by introspecting each extractor's
@property defs and TARGET_VARIABLES, plus running MISC.extract_all
on CO.0006.R06.00: H=100, T=73, A=19, M=151, UNION=161.

build_updated_data_dictionary.py + 1915C_Data_Dictionary_Updated.xlsx:
add canonical entries for the merged radio columns (costlimit,
local_eval, local_eval_instrument, sd_authority, sd_election,
spousal_impov_bc, statecontracts_mcos) and resolve typo'd column
names.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com> vrajesh1: I've read through and administered these changes
</commit_message>
<xml_diff>
--- a/docs/1915C_Data_Dictionary_Updated.xlsx
+++ b/docs/1915C_Data_Dictionary_Updated.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Variables'!$A$1:$K$168</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Waiver Data'!$A$1:$K$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Variables'!$A$1:$K$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Waiver Data'!$A$1:$K$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CSV-Only Columns'!$A$1:$E$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10">
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K168"/>
+  <dimension ref="A1:K169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4710,12 +4710,20 @@
           <t>Text Box</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v/>
-      </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="n">
-        <v/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Numeric (one or more)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Minimum number of services to qualify (text box).</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Free-text numeric entry from svapdxB6_1:elgEvalSvcMinQty. The state specifies the minimum count of waiver services an individual must require in the service plan in order to be determined to need waiver services. Almost always '1' in the corpus.</t>
+        </is>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
@@ -4757,7 +4765,7 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>1 = Directly by the Medicaid agency; 2 = By the operating agency specified in Appendix A; 3 = By an entity under contract with the Medicaid agency; 4 = Other</t>
+          <t>1 = Directly by the Medicaid agency; 2 = By the operating agency specified in Appendix A; 3 = By a government agency under contract with the Medicaid agency; 4 = Other</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
@@ -7672,8 +7680,53 @@
       </c>
       <c r="K168" s="5" t="inlineStr"/>
     </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>reeval_sched</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>Frequency of level-of-care reevaluations (Appendix B-6-g)</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>Radio Button</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>1 = Every three months; 2 = Every six months; 3 = Every twelve months; 4 = Other schedule</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>Reevaluation schedule (radio).</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>Merged radio variable from svapdxB6_1:elgRevalSchType. Emitted by the PDF acroform extractor; HTML and text extractors produce this via the radio-collapse layer over reeval_sched_3mo/_6mo/_12mo/_other.</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr"/>
+      <c r="I169" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J169" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K169" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K168"/>
+  <autoFilter ref="A1:K169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7684,7 +7737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8002,8 +8055,106 @@
       </c>
       <c r="K8" s="5" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>min_numservices</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Minimum number of waiver services required for an individual to be determined to need waiver services (Appendix B-6-a-i)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Text Box</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Numeric (one or more)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Minimum number of services to qualify (text box).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Free-text numeric entry from svapdxB6_1:elgEvalSvcMinQty. The state specifies the minimum count of waiver services an individual must require in the service plan in order to be determined to need waiver services. Almost always '1' in the corpus.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.0; 2.0; 5.0; 100.0; 4.0; 11.0; 12.0; 0.0; 48.0; 3.0; 6.0</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1065</v>
+      </c>
+      <c r="J9" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>numeric</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>reeval_sched</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Frequency of level-of-care reevaluations (Appendix B-6-g)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Radio Button</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>1 = Every three months; 2 = Every six months; 3 = Every twelve months; 4 = Other schedule</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Reevaluation schedule (radio).</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Merged radio variable from svapdxB6_1:elgRevalSchType. Emitted by the PDF acroform extractor; HTML and text extractors produce this via the radio-collapse layer over reeval_sched_3mo/_6mo/_12mo/_other.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr"/>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K8"/>
+  <autoFilter ref="A1:K10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>